<commit_message>
Update clic_data.xlsx with latest study statuses and notes
</commit_message>
<xml_diff>
--- a/clic_data.xlsx
+++ b/clic_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luxxx371\Box\Requests\Clic\Administration\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EEE9FFD-9A94-4005-9F3B-F1735852DFEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9154C786-D535-4D89-9BE7-15A77DB2C1BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Total Studies" sheetId="8" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2043" uniqueCount="363">
   <si>
     <t>Country</t>
   </si>
@@ -1767,7 +1767,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2130,13 +2130,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="27">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2147,7 +2160,35 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3323,7 +3364,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="38" t="s">
         <v>167</v>
       </c>
@@ -3352,7 +3393,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="142.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="71" t="s">
         <v>167</v>
       </c>
@@ -4166,10 +4207,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A54">
-    <cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="Associate">
+    <cfRule type="containsText" dxfId="26" priority="1" operator="containsText" text="Associate">
       <formula>NOT(ISERROR(SEARCH("Associate",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="2" operator="containsText" text="Full">
+    <cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="Full">
       <formula>NOT(ISERROR(SEARCH("Full",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5911,19 +5952,19 @@
   </sheetData>
   <autoFilter ref="A1:U25" xr:uid="{3D260CD3-4DAF-439E-9373-903363993C97}"/>
   <conditionalFormatting sqref="E2:S25">
-    <cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="Imputation">
+    <cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="Imputation">
       <formula>NOT(ISERROR(SEARCH("Imputation",E2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="2" operator="containsText" text="Not Applicable">
+    <cfRule type="containsText" dxfId="23" priority="2" operator="containsText" text="Not Applicable">
       <formula>NOT(ISERROR(SEARCH("Not Applicable",E2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="3" operator="containsText" text="Completed">
+    <cfRule type="containsText" dxfId="22" priority="3" operator="containsText" text="Completed">
       <formula>NOT(ISERROR(SEARCH("Completed",E2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="4" operator="containsText" text="Ongoing">
+    <cfRule type="containsText" dxfId="21" priority="4" operator="containsText" text="Ongoing">
       <formula>NOT(ISERROR(SEARCH("Ongoing",E2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="5" operator="containsText" text="Not started">
+    <cfRule type="containsText" dxfId="20" priority="5" operator="containsText" text="Not started">
       <formula>NOT(ISERROR(SEARCH("Not started",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5945,7 +5986,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -6076,11 +6117,11 @@
       <c r="C4" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="D4" s="34" t="s">
-        <v>157</v>
+      <c r="D4" s="31" t="s">
+        <v>156</v>
       </c>
       <c r="E4" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F4" s="108" t="s">
         <v>348</v>
@@ -6112,11 +6153,11 @@
       <c r="C5" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D5" s="34" t="s">
-        <v>157</v>
+      <c r="D5" s="31" t="s">
+        <v>156</v>
       </c>
       <c r="E5" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F5" s="108" t="s">
         <v>348</v>
@@ -6224,7 +6265,7 @@
         <v>156</v>
       </c>
       <c r="E8" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F8" s="108" t="s">
         <v>348</v>
@@ -6332,7 +6373,7 @@
         <v>156</v>
       </c>
       <c r="E11" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F11" s="108" t="s">
         <v>348</v>
@@ -6368,7 +6409,7 @@
         <v>156</v>
       </c>
       <c r="E12" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F12" s="108" t="s">
         <v>348</v>
@@ -6440,7 +6481,7 @@
         <v>156</v>
       </c>
       <c r="E14" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F14" s="108" t="s">
         <v>348</v>
@@ -6476,7 +6517,7 @@
         <v>156</v>
       </c>
       <c r="E15" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F15" s="108" t="s">
         <v>348</v>
@@ -6620,7 +6661,7 @@
         <v>156</v>
       </c>
       <c r="E19" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F19" s="108" t="s">
         <v>348</v>
@@ -6692,7 +6733,7 @@
         <v>156</v>
       </c>
       <c r="E21" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F21" s="108" t="s">
         <v>348</v>
@@ -6728,7 +6769,7 @@
         <v>156</v>
       </c>
       <c r="E22" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F22" s="108" t="s">
         <v>348</v>
@@ -6760,8 +6801,8 @@
       <c r="C23" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="D23" s="34" t="s">
-        <v>157</v>
+      <c r="D23" s="31" t="s">
+        <v>156</v>
       </c>
       <c r="E23" s="108" t="s">
         <v>348</v>
@@ -6800,7 +6841,7 @@
         <v>156</v>
       </c>
       <c r="E24" s="108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F24" s="108" t="s">
         <v>348</v>
@@ -6858,8 +6899,1038 @@
       </c>
       <c r="L25" s="28"/>
     </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="124" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" s="123" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E26" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L26" s="32"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="E2:K25">
+    <cfRule type="containsText" dxfId="19" priority="6" operator="containsText" text="Imputation">
+      <formula>NOT(ISERROR(SEARCH("Imputation",E2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="Not Applicable">
+      <formula>NOT(ISERROR(SEARCH("Not Applicable",E2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="17" priority="8" operator="containsText" text="Completed">
+      <formula>NOT(ISERROR(SEARCH("Completed",E2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="16" priority="9" operator="containsText" text="Ongoing">
+      <formula>NOT(ISERROR(SEARCH("Ongoing",E2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="10" operator="containsText" text="Not started">
+      <formula>NOT(ISERROR(SEARCH("Not started",E2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26:K26">
+    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Imputation">
+      <formula>NOT(ISERROR(SEARCH("Imputation",E26)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Not Applicable">
+      <formula>NOT(ISERROR(SEARCH("Not Applicable",E26)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Completed">
+      <formula>NOT(ISERROR(SEARCH("Completed",E26)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="Ongoing">
+      <formula>NOT(ISERROR(SEARCH("Ongoing",E26)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="Not started">
+      <formula>NOT(ISERROR(SEARCH("Not started",E26)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:K26" xr:uid="{A555EAE2-07F1-4F5A-B6E3-B3D53739CFEA}">
+      <formula1>"Completed, Ongoing,Not started,Not Applicable,Unknown,Done"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:L26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="35.28515625" customWidth="1"/>
+    <col min="3" max="6" width="26" customWidth="1"/>
+    <col min="7" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="57.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="101" t="s">
+        <v>154</v>
+      </c>
+      <c r="E1" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="F1" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="G1" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="K1" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="L1" s="27" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E2" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F2" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G2" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H2" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I2" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J2" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K2" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L2" s="32"/>
+    </row>
+    <row r="3" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F3" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G3" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H3" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I3" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J3" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K3" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L3" s="32"/>
+    </row>
+    <row r="4" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F4" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G4" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H4" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I4" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J4" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K4" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L4" s="32"/>
+    </row>
+    <row r="5" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F5" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G5" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H5" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I5" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J5" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K5" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L5" s="32"/>
+    </row>
+    <row r="6" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E6" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F6" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G6" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H6" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I6" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J6" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K6" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L6" s="32"/>
+    </row>
+    <row r="7" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E7" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F7" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G7" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H7" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I7" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J7" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K7" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L7" s="32"/>
+    </row>
+    <row r="8" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E8" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F8" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G8" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H8" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I8" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J8" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K8" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L8" s="32"/>
+    </row>
+    <row r="9" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E9" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F9" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G9" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H9" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I9" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J9" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K9" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L9" s="32"/>
+    </row>
+    <row r="10" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E10" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F10" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G10" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H10" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I10" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J10" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K10" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L10" s="32"/>
+    </row>
+    <row r="11" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E11" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F11" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G11" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H11" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I11" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J11" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K11" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L11" s="32"/>
+    </row>
+    <row r="12" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E12" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F12" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G12" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H12" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I12" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J12" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K12" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L12" s="32"/>
+    </row>
+    <row r="13" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E13" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F13" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G13" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H13" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I13" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J13" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K13" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L13" s="32"/>
+    </row>
+    <row r="14" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E14" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F14" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G14" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H14" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I14" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J14" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K14" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L14" s="32"/>
+    </row>
+    <row r="15" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E15" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F15" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G15" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H15" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I15" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J15" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K15" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L15" s="32"/>
+    </row>
+    <row r="16" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E16" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F16" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G16" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H16" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I16" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J16" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K16" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L16" s="32"/>
+    </row>
+    <row r="17" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E17" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F17" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G17" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H17" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I17" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J17" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K17" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L17" s="32"/>
+    </row>
+    <row r="18" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E18" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F18" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G18" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H18" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I18" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J18" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K18" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L18" s="32"/>
+    </row>
+    <row r="19" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E19" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F19" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G19" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H19" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I19" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J19" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K19" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L19" s="32"/>
+    </row>
+    <row r="20" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E20" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F20" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G20" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H20" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I20" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J20" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K20" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L20" s="32"/>
+    </row>
+    <row r="21" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>132</v>
+      </c>
+      <c r="C21" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="D21" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E21" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F21" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G21" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H21" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I21" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J21" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K21" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L21" s="32"/>
+    </row>
+    <row r="22" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="35" t="s">
+        <v>132</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E22" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F22" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G22" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H22" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I22" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J22" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K22" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L22" s="32"/>
+    </row>
+    <row r="23" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="C23" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="E23" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F23" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G23" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H23" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I23" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J23" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K23" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L23" s="32"/>
+    </row>
+    <row r="24" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="D24" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E24" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F24" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G24" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H24" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I24" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J24" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K24" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L24" s="32"/>
+    </row>
+    <row r="25" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="C25" s="30" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E25" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="F25" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G25" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H25" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I25" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J25" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K25" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L25" s="32"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="124" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" s="123" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="E26" s="108" t="s">
+        <v>349</v>
+      </c>
+      <c r="F26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="G26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="H26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="I26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="J26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="K26" s="108" t="s">
+        <v>348</v>
+      </c>
+      <c r="L26" s="32"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:K26">
     <cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="Imputation">
       <formula>NOT(ISERROR(SEARCH("Imputation",E2)))</formula>
     </cfRule>
@@ -6877,948 +7948,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:K25" xr:uid="{A555EAE2-07F1-4F5A-B6E3-B3D53739CFEA}">
-      <formula1>"Completed, Ongoing,Not started,Not Applicable,Unknown,Done"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="35.28515625" customWidth="1"/>
-    <col min="3" max="6" width="26" customWidth="1"/>
-    <col min="7" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="16" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" ht="57.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="27" t="s">
-        <v>121</v>
-      </c>
-      <c r="C1" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="101" t="s">
-        <v>154</v>
-      </c>
-      <c r="E1" s="27" t="s">
-        <v>152</v>
-      </c>
-      <c r="F1" s="27" t="s">
-        <v>153</v>
-      </c>
-      <c r="G1" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="H1" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="I1" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="J1" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="K1" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="L1" s="27" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E2" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F2" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G2" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H2" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I2" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J2" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K2" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L2" s="32"/>
-    </row>
-    <row r="3" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="D3" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E3" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F3" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G3" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H3" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I3" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J3" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K3" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L3" s="32"/>
-    </row>
-    <row r="4" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="D4" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="E4" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F4" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G4" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H4" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I4" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J4" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K4" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L4" s="32"/>
-    </row>
-    <row r="5" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>123</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="D5" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="E5" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F5" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G5" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H5" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I5" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J5" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K5" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L5" s="32"/>
-    </row>
-    <row r="6" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="D6" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E6" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F6" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G6" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H6" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I6" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J6" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K6" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L6" s="32"/>
-    </row>
-    <row r="7" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E7" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F7" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G7" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H7" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I7" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J7" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K7" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L7" s="32"/>
-    </row>
-    <row r="8" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>125</v>
-      </c>
-      <c r="C8" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E8" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F8" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G8" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H8" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I8" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J8" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K8" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L8" s="32"/>
-    </row>
-    <row r="9" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>125</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E9" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F9" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G9" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H9" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I9" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J9" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K9" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L9" s="32"/>
-    </row>
-    <row r="10" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>125</v>
-      </c>
-      <c r="C10" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="D10" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E10" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F10" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G10" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H10" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I10" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J10" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K10" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L10" s="32"/>
-    </row>
-    <row r="11" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="D11" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E11" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F11" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G11" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H11" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I11" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J11" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K11" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L11" s="32"/>
-    </row>
-    <row r="12" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B12" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="D12" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E12" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F12" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G12" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H12" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I12" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J12" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K12" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L12" s="32"/>
-    </row>
-    <row r="13" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>111</v>
-      </c>
-      <c r="D13" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E13" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F13" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G13" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H13" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I13" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J13" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K13" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L13" s="32"/>
-    </row>
-    <row r="14" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="D14" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E14" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F14" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G14" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H14" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I14" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J14" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K14" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L14" s="32"/>
-    </row>
-    <row r="15" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B15" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E15" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F15" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G15" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H15" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I15" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J15" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K15" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L15" s="32"/>
-    </row>
-    <row r="16" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="25" t="s">
-        <v>127</v>
-      </c>
-      <c r="C16" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="D16" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E16" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F16" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G16" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H16" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I16" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J16" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K16" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L16" s="32"/>
-    </row>
-    <row r="17" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B17" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="D17" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E17" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F17" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G17" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H17" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I17" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J17" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K17" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L17" s="32"/>
-    </row>
-    <row r="18" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B18" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="C18" s="30" t="s">
-        <v>115</v>
-      </c>
-      <c r="D18" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E18" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F18" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G18" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H18" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I18" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J18" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K18" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L18" s="32"/>
-    </row>
-    <row r="19" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>17</v>
-      </c>
-      <c r="D19" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E19" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F19" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G19" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H19" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I19" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J19" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K19" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L19" s="32"/>
-    </row>
-    <row r="20" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="29" t="s">
-        <v>137</v>
-      </c>
-      <c r="B20" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="C20" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E20" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F20" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G20" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H20" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I20" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J20" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K20" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L20" s="32"/>
-    </row>
-    <row r="21" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="35" t="s">
-        <v>132</v>
-      </c>
-      <c r="C21" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E21" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F21" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G21" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H21" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I21" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J21" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K21" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L21" s="32"/>
-    </row>
-    <row r="22" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="35" t="s">
-        <v>132</v>
-      </c>
-      <c r="C22" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="D22" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E22" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F22" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G22" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H22" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I22" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J22" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K22" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L22" s="32"/>
-    </row>
-    <row r="23" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="25" t="s">
-        <v>133</v>
-      </c>
-      <c r="C23" s="30" t="s">
-        <v>118</v>
-      </c>
-      <c r="D23" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="E23" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F23" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G23" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H23" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I23" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J23" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K23" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L23" s="32"/>
-    </row>
-    <row r="24" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="29" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="C24" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="D24" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E24" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F24" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G24" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H24" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I24" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J24" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K24" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L24" s="32"/>
-    </row>
-    <row r="25" spans="1:12" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="29" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="C25" s="30" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="E25" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="F25" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="G25" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="H25" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="I25" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="J25" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="K25" s="108" t="s">
-        <v>348</v>
-      </c>
-      <c r="L25" s="32"/>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="E2:K25">
-    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="Imputation">
-      <formula>NOT(ISERROR(SEARCH("Imputation",E2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="Not Applicable">
-      <formula>NOT(ISERROR(SEARCH("Not Applicable",E2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="Completed">
-      <formula>NOT(ISERROR(SEARCH("Completed",E2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="Ongoing">
-      <formula>NOT(ISERROR(SEARCH("Ongoing",E2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="Not started">
-      <formula>NOT(ISERROR(SEARCH("Not started",E2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:K25" xr:uid="{AD093F45-6044-45B6-A91C-B146170D7F21}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:K26" xr:uid="{AD093F45-6044-45B6-A91C-B146170D7F21}">
       <formula1>"Completed, Ongoing,Not started,Not Applicable,Unknown,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9366,19 +9496,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:I51">
-    <cfRule type="beginsWith" dxfId="4" priority="1" operator="beginsWith" text="Complete">
+    <cfRule type="beginsWith" dxfId="9" priority="1" operator="beginsWith" text="Complete">
       <formula>LEFT(C2,LEN("Complete"))="Complete"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Planned">
+    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="Planned">
       <formula>NOT(ISERROR(SEARCH("Planned",C2)))</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="2" priority="3" operator="beginsWith" text="Incomplete">
+    <cfRule type="beginsWith" dxfId="7" priority="3" operator="beginsWith" text="Incomplete">
       <formula>LEFT(C2,LEN("Incomplete"))="Incomplete"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Not Applicable">
+    <cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="Not Applicable">
       <formula>NOT(ISERROR(SEARCH("Not Applicable",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="Unknown">
+    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="Unknown">
       <formula>NOT(ISERROR(SEARCH("Unknown",C2)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Update app code, report, and clic_data file
</commit_message>
<xml_diff>
--- a/clic_data.xlsx
+++ b/clic_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luxxx371\Box\Requests\Clic\Administration\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B1CD1A7-15A0-45F6-B49C-9DC725A211D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061E6B36-B134-4CFD-BAF7-AE28F4AAF8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Total Studies" sheetId="8" r:id="rId1"/>
@@ -1182,9 +1182,6 @@
     <t>Planned</t>
   </si>
   <si>
-    <t>Soutsh Mexican study</t>
-  </si>
-  <si>
     <t>Juan Carlos Núñez-Enríquez</t>
   </si>
   <si>
@@ -1192,6 +1189,9 @@
   </si>
   <si>
     <t>SMS</t>
+  </si>
+  <si>
+    <t>South Mexican study</t>
   </si>
 </sst>
 </file>
@@ -3540,13 +3540,13 @@
         <v>32</v>
       </c>
       <c r="D31" s="70" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>169</v>
       </c>
       <c r="F31" s="127" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G31" s="74" t="s">
         <v>229</v>
@@ -3555,7 +3555,7 @@
         <v>5</v>
       </c>
       <c r="I31" s="70" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -9011,7 +9011,7 @@
         <v>32</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C25" s="120" t="s">
         <v>5</v>

</xml_diff>